<commit_message>
Optimize UniversityCourse export with searchable names and descriptions
</commit_message>
<xml_diff>
--- a/tcu/tcu_data.xlsx
+++ b/tcu/tcu_data.xlsx
@@ -451,17 +451,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aga Khan University (AKU)</t>
+          <t>Aga Khan University (AKU) Abdulrahman Al- Sumait University (SUMAIT) Archbishop Mihayo University College of Tabora (AMUCTA)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>University University University College</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Private Private Private</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -478,17 +478,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ardhi University (ARU)</t>
+          <t>Ardhi University (ARU) Arusha Technical College (ATC) Catholic University of Health and Allied Sciences (CUHAS) Name of Institution Center for Foreign Relations (CFR) College of African Wildlife</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>University Non- University University Type of Institution Non- University Non-</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Private Ownership Status Public Public</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -505,12 +505,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Management Mweka (CAWM) College of Business</t>
+          <t>Management Mweka (CAWM) College of Business Education (CBE) Dar es Salaam</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>University Non-</t>
+          <t>University Non- University</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -586,17 +586,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>College of Business Education (CBE) Mbeya</t>
+          <t>College of Business Education (CBE) Mbeya Dar es Salaam Institute of Technology (DIT) Dar es Salaam Institute of Technology (DIT)-Mwanza Campus</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University Non- University Non- University</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Public</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dar es Salaam Maritime Institute (DMI)</t>
+          <t>Dar es Salaam Maritime Institute (DMI) Dar es Salaam Tumaini University (DarTU) Dar es Salaam University College of Education (DUCE)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University University University College</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Private Public</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -640,17 +640,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Eastern Africa Statistical Training Centre (EASTC)</t>
+          <t>Eastern Africa Statistical Training Centre (EASTC) Institute of Accountancy Arusha (IAA) Institute of Accountancy Arusha (IAA) Dar es Salaam Campus</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University Non- University Non- University</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Public</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -667,17 +667,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Institute of Adult Education (IAE)</t>
+          <t>Institute of Adult Education (IAE) Name of Institution</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University Type of Institution</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Ownership Status</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Management (IFM)- Dodoma Institute of Finance</t>
+          <t>Management (IFM)- Dodoma Institute of Finance Management (IFM)- Mwanza</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>University Non-</t>
+          <t>University Non- University</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -748,17 +748,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Institute of Finance Management (IFM)-Simiyu</t>
+          <t>Institute of Finance Management (IFM)-Simiyu Institute of Public Administration (IPA) Institute of Rural</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University Non- University Non-</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Public</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -775,12 +775,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Development Planning (IRDP) Institute of Rural</t>
+          <t>Development Planning (IRDP) Institute of Rural Development Planning (IRDP)-Mwanza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>University Non-</t>
+          <t>University Non- University</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -829,17 +829,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Institute of Social Work- Kisangara Campus (ISW)</t>
+          <t>Institute of Social Work- Kisangara Campus (ISW) Institute of Tax Administration (ITA) Jordan University College (JUCo) Kairuki University (KU) Kampala International University in Tanzania</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University Non- University University College University University</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Private Private Private</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -856,17 +856,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>(KIUT) Karume Institute of</t>
+          <t>(KIUT) Karume Institute of Science and Technology (KIST) Name of Institution</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Non-</t>
+          <t>Non- University Type of Institution</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Ownership Status</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -883,12 +883,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kizumbi Institute of</t>
+          <t>Kizumbi Institute of Cooperative Business Education (KICoB)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>University Campus Institute</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -910,17 +910,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Local Government Training Institute (LGTI)</t>
+          <t>Local Government Training Institute (LGTI) Marian University College (MARUCo) Mbeya University of</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University University College University</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Private Public</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -991,17 +991,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Technical Education (MUST – MCCTE) Mkwawa University</t>
+          <t>Technical Education (MUST – MCCTE) Mkwawa University College of Education (MUCE) Moshi Cooperative University (MoCU) MS Training Centre for</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>University College University Non-</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Private</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1018,17 +1018,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Development Cooperation (MS-TCDC) Muhimbili University of</t>
+          <t>Development Cooperation (MS-TCDC) Muhimbili University of Health and Allied Sciences (MUHAS) Muslim University of Morogoro (MUM) Mwalimu Nyerere Memorial Academy (MNMA) Name of Institution</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>University University</t>
+          <t>University University University Non- University Type of Institution</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Private Public Ownership Status</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Memorial Academy (MNMA)- Pemba Campus Mwalimu Nyerere University of Agriculture and Technology</t>
+          <t>Memorial Academy (MNMA)- Pemba Campus Mwalimu Nyerere University of Agriculture and Technology (MNUAT), Musoma</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1126,17 +1126,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Mwenge Catholic University (MWECAU)</t>
+          <t>Mwenge Catholic University (MWECAU) Mzumbe University (MU) Mzumbe University Dar es</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>University University University</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Private Public Public</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Salaam Campus College (MUDCCo) Mzumbe University</t>
+          <t>Salaam Campus College (MUDCCo) Mzumbe University Mbeya Campus College (MUMCCo)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Campus College University</t>
+          <t>Campus College University Campus College</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1234,17 +1234,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ruaha Catholic University (RUCU)</t>
+          <t>Ruaha Catholic University (RUCU) Sokoine University of Agriculture (SUA) Sokoine University of Agriculture(SUA) - Mizengo Pinda Campus College St. Augustine University of Tanzania (SAUT) St. Augustine University of</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>University University University Campus College University University</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Private Public Public Private Private</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1261,17 +1261,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Tanzania (SAUT) -Arusha Centre St. Francis University</t>
+          <t>Tanzania (SAUT) -Arusha Centre St. Francis University Name of Institution Ifakara St. John’s University of Tanzania (SJUT) St. Joseph University</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Centre University</t>
+          <t>Centre University Type of Institution University University</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Private Ownership Status Private Private</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1288,17 +1288,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>College of Health and Allied Sciences (SJCHAS) St. Joseph University</t>
+          <t>College of Health and Allied Sciences (SJCHAS) St. Joseph University College of Engineering and Technology (SJCET) State University of Zanzibar (SUZA) Stella Maris Mtwara</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>University University University</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Private Public Private</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1315,12 +1315,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>University College (STeMMUCo) Tanzania Institute of</t>
+          <t>University College (STeMMUCo) Tanzania Institute of Accountancy (TIA), Dar es Salaam</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>College Non-</t>
+          <t>College Non- University</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1342,17 +1342,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tanzania Institute of Accountancy (TIA), Mbeya</t>
+          <t>Tanzania Institute of Accountancy (TIA), Mbeya Tanzania Institute of Accountancy (TIA), Mtwara Tanzania Institute of</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University Non- University Non-</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Public</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1396,17 +1396,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Accountancy (TIA), Singida Tanzania Institute of</t>
+          <t>Accountancy (TIA), Singida Tanzania Institute of Accountancy (TIA), Kigoma Tanzania Institute of Accountancy (TIA), Tanga Tanzania Public Service</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>University Non-</t>
+          <t>University Non- University Non- University Non-</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Public Public</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1423,17 +1423,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>College (TPSC), Dar es Salaam Campus Tanzania Institute of Project</t>
+          <t>College (TPSC), Dar es Salaam Campus Tanzania Institute of Project Management (TIPM), Dar es Salaam Name of Institution Community Development (TICD)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>University Non-</t>
+          <t>University Non- University Type of Institution University</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Private Ownership Status</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1666,17 +1666,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Water Institute (WI)</t>
+          <t>Water Institute (WI) Activity</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Non- University</t>
+          <t>Non- University Responsible</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Public Date</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Science with Education Bachelor of Arts in Counselling Psychology</t>
+          <t>Bachelor of Arts in Science with Education Counselling Psychology</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Education Bachelor of Business Administration</t>
+          <t>Bachelor of Business Education Administration</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Bachelor of Arts in</t>
+          <t>Bachelor of Arts in Environment and Natural Resources</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>A-level. Two Principal level passes in any of the following subjects: Physics, Advanced Mathematics, Chemistry, Biology, Computer Science or Geography. One of the two principal level passes</t>
+          <t>A-level. Two Principal level passes in any of the following subjects: Physics, Advanced Mathematics, Chemistry, Biology, Computer Science or Geography. One of the two principal level passes . Mathematics or Basic Applied Mathematics at A-level or a</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Planning Bachelor of Science in Land Management and Valuation</t>
+          <t>Bachelor of Science Planning in Land Management and Valuation</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Bachelor of Science in</t>
+          <t>Bachelor of Science in Engineerig</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Mathematics and “D” grade in English Language at O-Level. Two Principal level passes in any of the following subjects: Physics, Advanced Mathematics, Chemistry, Computer Science</t>
+          <t>Mathematics and “D” grade in English Language at O-Level. Two Principal level passes in any of the following subjects: Physics, Advanced Mathematics, Chemistry, Computer Science least a subsidiary level pass in Advanced Mathematics or Basic</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Regional Development Planning</t>
+          <t>Bachelor of Science in Regional Development Planning Finance and Investment</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Mathematics and “D” grade in English Language at O-Level. Two principal level passes in any of the following subjects: Physics, Chemistry, Biology, Advanced Mathematics, Geography, Economics, Commerce, Computer Science or Accountancy. In addition, an applicant must have at least a subsidiary level pass in Basic Applied Mathematics or D grade in Advanced Mathematics at A-level or a minimum of “ C ”</t>
+          <t>Mathematics and “D” grade in English Language at O-Level. Two principal level passes in any of the following subjects: Physics, Chemistry, Biology, Advanced Mathematics, Geography, Economics, Commerce, Computer Science or Accountancy. In addition, an applicant must have at least a subsidiary level pass in Basic Applied Mathematics or D grade in Advanced Mathematics at A-level or a minimum of “ C ” grade in Basic Mathematics at O-Level. Geography, Advanced Mathematics, Physics, Biology or Chemistry. In addition, an applicant must have at least a subsidiary level pass in Advanced Mathematics or Basic Applied Mathematics at A-level or a minimum of “ D ” grade in Basic Mathematics and a minimum of ‘D’ grade in English Language at</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Level. A principal pass in Economics and a principal pass in any of</t>
+          <t>Level. A principal pass in Economics and a principal pass in any of In addition, an applicant must have at least a subsidiary level pass in Advanced Mathematics or Basic Applied Mathematics at A-level or a minimum of “D” grade in Basic Mathematics at</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Civil Engineering</t>
+          <t>Bachelor of Science in Civil Engineering Science in Accounting and Finance</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>grade of "C" in Basic Mathematics at O-Level. Two Principal level passes in the following subjects: Advanced Mathematics and Physics. Those without at least a Subsidiary pass in Chemistry at A-Level must have a</t>
+          <t>grade of "C" in Basic Mathematics at O-Level. Two Principal level passes in the following subjects: Advanced Mathematics and Physics. Those without at least a Subsidiary pass in Chemistry at A-Level must have a minimum of “C”grade in Chemistry at O-level. Mathematics, Geography, History, Physics, Biology or Chemistry. In addition, an applicant must have at least a subsidiary level pass in Advanced Mathematics or Basic Applied Mathematics at A-level or a minimum of “D” grade in Basic Mathematics and a minimum of ‘ D ’ grade in English Language at O-Level or a pass in English/English Literature at</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Studies Bachelor of Science in Geographical Information Systems</t>
+          <t>Bachelor of Studies Science in Geographical Information Systems</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Economics Bachelor of Science in Environmental Laboratory Science and Technology</t>
+          <t>Bachelor of Economics Science in Environmental Laboratory Science and Technology</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Computer</t>
+          <t>Bachelor of Science in Computer Networks</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>grade in Basic Mathematics at O-Level. Two principal level passes in any of the following subjects: Advanced Mathematics, Physics, Geography, Biology, Chemistry,</t>
+          <t>grade in Basic Mathematics at O-Level. Two principal level passes in any of the following subjects: Advanced Mathematics, Physics, Geography, Biology, Chemistry, Mathematics at A-level and a minimum grade of "C" in Basic</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Maintenance Bachelor of Science in Data Science and Artificial Intelligence</t>
+          <t>Bachelor of Science Maintenance in Data Science and Artificial Intelligence</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Computer Science Bachelor Degree in</t>
+          <t>Bachelor Degree in Computer Science</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Information Technology Bachelor Degree in</t>
+          <t>Bachelor Degree in Information Technology</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Bachelor Degree in</t>
+          <t>Bachelor Degree in Mechanical Engineering</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Education Bachelor of Business Administration</t>
+          <t>Bachelor of Business Education Administration</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>English an applicant must have a minimum of D grade in English at O-Level. Two principal passes in the following subjects: History, Geography, Economics, Commerce, Accountancy, Physics,</t>
+          <t>English an applicant must have a minimum of D grade in English at O-Level. Two principal passes in the following subjects: History, Geography, Economics, Commerce, Accountancy, Physics, Advanced Mathematics an applicant must have a subsidiary “ ” . pass in Advanced Mathematics/Basic Applied Mathematics</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Development Bachelor of Arts in Social Work</t>
+          <t>Bachelor of Arts in Development Social Work</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Relations and Diplomacy Bachelor Degree in Governance and Strategic</t>
+          <t>Diplomacy Relations and Bachelor Degree in Governance and Strategic</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Waste Management Bachelor Degree in Natural Resources</t>
+          <t>Bachelor Degree in Waste Management Natural Resources</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Bachelor Degree in Marketing</t>
+          <t>Bachelor Degree in Marketing Supplies Chain</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3495,7 +3495,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Chemistry, Biology, Computer Science, or Fine Arts. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, Literature, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture,</t>
+          <t>Chemistry, Biology, Computer Science, or Fine Arts. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, Literature, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. Geography, Physics, English, Kiswahili, History, Chemistry,</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Metrology and Standardization</t>
+          <t>Bachelor Degree in Management Metrology and Standardization</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Education Bachelor Degree of Business Administration in Human Resources</t>
+          <t>Bachelor Degree of Education Business Administration in Human Resources Management Management</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Geography, Physics, Chemistry, Biology, History or English. Two Principal passes in the following subjects; Accountancy, Economics, Commerce, Advanced Mathematics, Geography, Physics, English, Kiswahili, History, Chemistry or Biology.</t>
+          <t>Geography, Physics, Chemistry, Biology, History or English. Two Principal passes in the following subjects; Accountancy, Economics, Commerce, Advanced Mathematics, Geography, Physics, English, Kiswahili, History, Chemistry or Biology. Commerce, Agriculture, English, History,</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Bachelor Degree in Banking and Finance</t>
+          <t>Bachelor Degree in Banking and Finance Management</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Basic Mathematics at O Level Two principal passes in the following subjects: Biology, Chemistry, Physics, Geography, Agriculture, Nutrition, Advanced Mathematics, Accountancy, Commerce, English Language, Kiswahili or Economics. If one of the principal passes is not in ’ Advanced Mathematics, an applicant must have at least a Pass in</t>
+          <t>Basic Mathematics at O Level Two principal passes in the following subjects: Biology, Chemistry, Physics, Geography, Agriculture, Nutrition, Advanced Mathematics, Accountancy, Commerce, English Language, Kiswahili or Economics. If one of the principal passes is not in ’ Advanced Mathematics, an applicant must have at least a Pass in Basic Mathematics at O Level Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -3699,7 +3699,11 @@
           <t>College of Business Education (CBE), Dar es Salaam</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Bachelor degree in Digital Marketing</t>
+        </is>
+      </c>
       <c r="C124" t="inlineStr">
         <is>
           <t>CBD14</t>
@@ -3722,7 +3726,11 @@
           <t>College of Business Education (CBE), Dar es Salaam</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Bachelor Degree in Economics and Finance</t>
+        </is>
+      </c>
       <c r="C125" t="inlineStr">
         <is>
           <t>CBD15</t>
@@ -3745,7 +3753,11 @@
           <t>College of Business Education (CBE), Dar es Salaam</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Bachelor Degree in Logistics and Transport</t>
+        </is>
+      </c>
       <c r="C126" t="inlineStr">
         <is>
           <t>CBD16</t>
@@ -3768,7 +3780,11 @@
           <t>College of Business Education (CBE), Dar es Salaam</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Bachelor Degree in Entrepreneurship and Innovation</t>
+        </is>
+      </c>
       <c r="C127" t="inlineStr">
         <is>
           <t>CBD17</t>
@@ -3820,7 +3836,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Education Bachelor of Commerce and Accountancy with</t>
+          <t>Bachelor of Commerce Education and Accountancy with</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3847,17 +3863,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Education Bachelor’s Degree of Business Administration (Double</t>
+          <t>Bachelor’s Degree of Education Business Administration (Double Bachelor’s Degree in Degree) Digital and Technology Solutions Management</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>CBD20</t>
+          <t>CBD20 CBD21</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Computer studies, Commerce, Accounts and Physics. Two principal passes in the following subjects: Accountancy, Economics, Commerce, Advanced Mathematics, Geography, Physics, English, Agriculture, Nutrition, Chemistry, Biology, Computer Science.</t>
+          <t>Computer studies, Commerce, Accounts and Physics. Two principal passes in the following subjects: Accountancy, Economics, Commerce, Advanced Mathematics, Geography, Physics, English, Agriculture, Nutrition, Chemistry, Biology, Computer Science. Two principal passes in the following subjects: Advanced Mathematics, Chemistry, Geography, Economics, Biology, Computer studies, Commerce, Accounts and Physics.</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -3928,7 +3944,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Administration Bachelor Degree in Marketing</t>
+          <t>Bachelor Degree in Administration Marketing Procurement and Supplies Management</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3938,7 +3954,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>History, Agriculture, Nutrition, Chemistry or Biology. Two principal passes in the following subjects: History, Geography, Kiswahili, English, Literature, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics,</t>
+          <t>History, Agriculture, Nutrition, Chemistry or Biology. Two principal passes in the following subjects: History, Geography, Kiswahili, English, Literature, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. Geography, Kiswahili, English, Literature, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics,</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -4009,7 +4025,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Technology Bachelor Degree of Business</t>
+          <t>Bachelor Degree of Technology Business Records and</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -4019,7 +4035,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Economics. Two principal passes in the following subjects: History, Geography, Kiswahili, English, Literature, French, Arabic,</t>
+          <t>Economics. Two principal passes in the following subjects: History, Geography, Kiswahili, English, Literature, French, Arabic, Computer Science or Nutrition.</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -4036,7 +4052,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Archives Management Bachelor Degree of Business Administration in</t>
+          <t>Bachelor Degree of Archives Management Business Administration in</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -4063,7 +4079,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Human Resources Management Bachelor of Accountancy and Taxation</t>
+          <t>Bachelor of Human Resources Management Accountancy and Taxation</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -4144,7 +4160,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Management Bachelor of Logistics and Transport</t>
+          <t>Bachelor of Management Logistics and Transport</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -4171,7 +4187,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Management Bachelor of Accountancy and Finance</t>
+          <t>Bachelor of Management Accountancy and Finance</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -4279,7 +4295,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Management Bachelor</t>
+          <t>Bachelor Management Studies with</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -4289,7 +4305,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography,</t>
+          <t>Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Mathematics, Agriculture, Computer Science or Nutrition.</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -4306,7 +4322,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Education Bachelor Degree in Marketing</t>
+          <t>Bachelor Degree Education in Marketing</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -4360,7 +4376,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Accounting and Finance</t>
+          <t>Bachelor Degree in Management Accounting and Finance</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4414,7 +4430,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Bachelor Degree</t>
+          <t>Bachelor Degree Logistic</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -4424,7 +4440,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Advanced</t>
+          <t>Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Advanced Computer Science or Nutrition.</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -4441,7 +4457,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree of Marketing in Tourism and</t>
+          <t>Bachelor Degree Management of Marketing in Tourism and</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -4603,7 +4619,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Engineering in Civil Engineering Bachelor of Engineering in</t>
+          <t>Bachelor of Engineering in Civil Engineering Engineering in</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4630,7 +4646,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Computer Engineering Bachelor of Engineering in</t>
+          <t>Bachelor of Computer Engineering Engineering in</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -4657,7 +4673,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Electrical Engineering Bachelor of Engineering in Electronics and</t>
+          <t>Bachelor of Engineering Electrical Engineering in Electronics and</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4684,7 +4700,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Telecommunication Engineering Bachelor of Engineering in Mechanical</t>
+          <t>Bachelor of Telecommunication Engineering Engineering in Mechanical</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4738,7 +4754,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Gas Engineering Bachelor of Technology in Laboratory Science</t>
+          <t>Bachelor of Technology Gas Engineering in Laboratory Science</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4792,7 +4808,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Engineering Bachelor of Engineering in Biomedical</t>
+          <t>Bachelor of Engineering Engineering in Biomedical</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -4873,7 +4889,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>and Nautical Science Bachelor Degree in Marine Engineering</t>
+          <t>Bachelor Degree in and Nautical Science Marine Engineering</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4900,7 +4916,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Technology Bachelor Degree in Shipping and Logistics</t>
+          <t>Bachelor Degree in Technology Shipping and Logistics</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4927,7 +4943,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Naval Architecture and Offshore</t>
+          <t>Bachelor Degree in Management Naval Architecture and Offshore Engineering Supply Chain</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4937,7 +4953,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>History, Literature or English. Two principal passes in the following subjects: Advanced Mathematics, Physics or Chemistry.</t>
+          <t>History, Literature or English. Two principal passes in the following subjects: Advanced Mathematics, Physics or Chemistry. Biology, Accountancy, Geography, History,</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -4954,7 +4970,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Transport and Supply Chain Management</t>
+          <t>Bachelor Degree in Management Transport and Supply Chain Management</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -5008,7 +5024,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Engineering Bachelor Degree in</t>
+          <t>Bachelor Degree in Engineering</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -5035,7 +5051,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Oil and Gas Engineering Bachelor Degree in</t>
+          <t>Bachelor Degree in Oil and Gas Engineering</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -5197,17 +5213,17 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Bachelor of Information Systems</t>
+          <t>Bachelor of Information Systems Management Bachelor of Human Bachelor of Arts with Education Resources Management</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>TD005</t>
+          <t>TD005 TD006 TD007</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics,</t>
+          <t>Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: English, History, Kiswahili, Geography, Literature or Economics. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -5234,7 +5250,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce,</t>
+          <t>Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Nutrition. If one of the principal passes is not in English an applicant MUST HAVE subsidiary pass in</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -5332,7 +5348,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Computing (Evening Session) Bachelor of Theology</t>
+          <t>Bachelor of Computing (Evening Session) Theology</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -5413,7 +5429,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Education (evening) Bachelor of Business</t>
+          <t>Bachelor of Education (evening) Business</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -5440,7 +5456,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Administration in Marketing Bachelor of Business</t>
+          <t>Bachelor of Administration in Marketing Business</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -5467,7 +5483,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Administration in Accounting Bachelor of Science in Computer Science (Cybersecurity)</t>
+          <t>Bachelor of Science Administration in Accounting in Computer Science (Cybersecurity)</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -5548,7 +5564,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Education Bachelor of Arts in</t>
+          <t>Bachelor of Education Arts in</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -5656,7 +5672,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Bachelor Degree in Agricultural Statistics and Economics</t>
+          <t>Bachelor Degree in Agricultural Statistics and Economics Science in Actuarial</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -5666,7 +5682,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>required. Two principal passes in the following subjects: Advanced Mathematics, Physics, Chemistry, Biology, Accountancy, Agriculture, Geography, Economics, Computers, Commerce, Nutrition, Business Studies, Education, Food &amp; Nutrition and Computer Science. If one of the principal passes is not in ‘’D’’ Advanced Mathematics, a Subsidiary pass in Basic Applied Mathematics or a minimum of grade in Mathematics at O-</t>
+          <t>required. Two principal passes in the following subjects: Advanced Mathematics, Physics, Chemistry, Biology, Accountancy, Agriculture, Geography, Economics, Computers, Commerce, Nutrition, Business Studies, Education, Food &amp; Nutrition and Computer Science. If one of the principal passes is not in ‘’D’’ Advanced Mathematics, a Subsidiary pass in Basic Applied Mathematics or a minimum of grade in Mathematics at O- Level is required. the following subjects; Economics, Geography, Commerce, Accountancy, Business Studies, Physics, Chemistry, Biology,</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -5737,7 +5753,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Bachelor of Computer</t>
+          <t>Bachelor of Computer Science Technology</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -5747,7 +5763,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Computer Science or Nutrition. Two principal passes in the following subjects: Physics, Chemistry, Biology, Computer Studies, Agriculture,</t>
+          <t>Computer Science or Nutrition. Two principal passes in the following subjects: Physics, Chemistry, Biology, Computer Studies, Agriculture, Geography or Advanced Mathematics. Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. If one of the principal passes is not in Advanced Mathematics an applicant must have at least a subsidiary pass or a minimum of “D”</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -5791,7 +5807,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Management Bachelor of Economics and Finance</t>
+          <t>Bachelor of Economics Management and Finance</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -5828,7 +5844,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Mathematics. Two principal passes in the following subjects:</t>
+          <t>Mathematics. Two principal passes in the following subjects: the principal passes is not in Advanced Mathematics an “ ” applicant must have at least a subsidiary pass or a</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -5926,7 +5942,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Bachelor of Education with Computer Science</t>
+          <t>Bachelor of Education with Computer Science with Apprenticeship</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5936,7 +5952,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>grade in Mathematics at O-Level. Two principal passes in the following subjects: Physics, Chemistry, Biology, compute science, Agriculture, Geography or Advanced Mathematics. If one of the principal passes is not in Advanced Mathematics an “ ” applicant must have at least a subsidiary pass or a</t>
+          <t>grade in Mathematics at O-Level. Two principal passes in the following subjects: Physics, Chemistry, Biology, compute science, Agriculture, Geography or Advanced Mathematics. If one of the principal passes is not in Advanced Mathematics an “ ” applicant must have at least a subsidiary pass or a minimum of C grade in Mathematics at O-Level. Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture,</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -6169,7 +6185,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>and Project Management Bachelor of Records and Information Management</t>
+          <t>Bachelor of Records and and Project Management Information Management</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -6412,7 +6428,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Computer Science Bachelor Degree in Information Technology</t>
+          <t>Bachelor Degree in Computer Science Information Technology</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -6520,7 +6536,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Adult and Continuing Education Bachelor Degree in Adult Education and</t>
+          <t>Bachelor Degree in Adult and Continuing Education Adult Education and</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -6547,7 +6563,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Community Development Bachelor Degree in Adult EducatioOnDaLnd</t>
+          <t>Bachelor Degree in Community Development Adult EducatioOnDaLnd</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6574,7 +6590,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Community Development ( ) Bachelor DeOgDreLe in</t>
+          <t>Bachelor DeOgDreLe in Community Development ( )</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -6790,7 +6806,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Science Bachelor of Science in Actuarial Sciences</t>
+          <t>Bachelor of Science Science in Actuarial Sciences</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -6898,7 +6914,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Security Bachelor of Computer Network</t>
+          <t>Bachelor of Security Computer Network</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -7114,7 +7130,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Bachelor Degree in International Relations and Diplomacy</t>
+          <t>Diplomacy Bachelor Degree in International Relations and</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -7303,7 +7319,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Planning Bachelor Degree in Regional Development Planning</t>
+          <t>Bachelor Degree in Planning Regional Development Planning</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -7357,7 +7373,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Bachelor Degree in Urban Development</t>
+          <t>Bachelor Degree in Urban Development Management</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -7367,7 +7383,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Computer Science. Two principal passes in the following subjects: Geography, Biology, Agriculture, Chemistry, Arabic, Physics, History,</t>
+          <t>Computer Science. Two principal passes in the following subjects: Geography, Biology, Agriculture, Chemistry, Arabic, Physics, History, Economics, Computer Science, Chinese, Physical Education</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -7448,7 +7464,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Education and Chinese. Two principal passes in the following subjects: Economics, Geography, History, Commerce, Accounting, Advanced</t>
+          <t>Education and Chinese. Two principal passes in the following subjects: Economics, Geography, History, Commerce, Accounting, Advanced English Language, Literature, Physics, Chemistry,</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -7529,7 +7545,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Chinese, Physical Education or Advanced Mathematics. Two Principal level passes in any of the following subjects: Geography, Economics, Advanced Mathematics, History, English Literature, Commerce, Accountancy, Physics,</t>
+          <t>Chinese, Physical Education or Advanced Mathematics. Two Principal level passes in any of the following subjects: Geography, Economics, Advanced Mathematics, History, English Literature, Commerce, Accountancy, Physics, “ ” Advanced Mathematics or Basic Applied Mathematics at A- ‘ ’ level or a minimum of C grade in Basic Mathematics and</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -7600,7 +7616,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Bachelor Degree in</t>
+          <t>Bachelor Degree in Administration</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -7610,7 +7626,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Mathematics and English at O- level. Two principal passes in the following subjects: History,</t>
+          <t>Mathematics and English at O- level. Two principal passes in the following subjects: History, principals is not Advanced Mathematics an applicant must “ ” have a subsidiary pass in Advanced Mathematics/Basic Applied Mathematics at A- Level or a D grade in Basic</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -7789,7 +7805,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Social Work</t>
+          <t>Bachelor Degree in Management Social Work</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -7816,7 +7832,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Bachelor Degree in Human Resource Management</t>
+          <t>Bachelor Degree in Human Resource Management Administration</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -7826,7 +7842,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>or Nutrition Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science</t>
+          <t>or Nutrition Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -8069,7 +8085,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Science or Nutrition. Two Principal passes in the following subjects: History,</t>
+          <t>Science or Nutrition. Two Principal passes in the following subjects: History, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition OR Foundation Certificate of the OUT</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -8275,17 +8291,17 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Management Bachelor of Science in</t>
+          <t>Bachelor of Management Science in Bachelor of Computer</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>JC013</t>
+          <t>JC013 KUC01</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Physics, Chemistry, Biology, Computer Studies, Agriculture, Geography</t>
+          <t>Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Physics, Chemistry, Biology, Computer Studies, Agriculture, Geography Physics, Chemistry, Biology, Computer Studies,</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -8302,7 +8318,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Science Bachelor of Information Technology</t>
+          <t>Bachelor of Science Information Technology</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -8366,7 +8382,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic,</t>
+          <t>Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Computer Science or Nutrition. If one of the principal passes is not in English and History at A-Level, an applicant must have a minimum of “D” grade in English</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -8410,7 +8426,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Education Bachelor of Public Administration</t>
+          <t>Bachelor of Public Education Administration</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -8518,7 +8534,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Bachelor of Business Administration (Marketing)</t>
+          <t>Bachelor of Business Administration (Marketing) (Procurement)</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -8528,7 +8544,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture,</t>
+          <t>Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture,</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -8626,7 +8642,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Medicine Bachelor of Science in Nursing</t>
+          <t>Bachelor of Medicine Science in Nursing</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -8680,17 +8696,17 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Bachelor of Engineering in Aircraft Maintenance</t>
+          <t>Bachelor of Engineering in Aircraft Maintenance Bachelor of Electrical Bachelor of Civil Engineering</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>KIS01</t>
+          <t>KIS01 KIS03 KIS04</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Two principal passes in Advanced Mathematics and Physics. Applicants without a principal pass in Chemistry must have at least a subsidiary pass in Chemistry at A-Level or a credit pass in Chemistry at</t>
+          <t>Two principal passes in Advanced Mathematics and Physics. Applicants without a principal pass in Chemistry must have at least a subsidiary pass in Chemistry at A-Level or a credit pass in Chemistry at O-Level. In addition, an applicant must have a credit in Physics or Mathematics at O-Level. Two principal passes in Physics and Advanced Mathematics. Two principal passes in Physics and Advanced</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -8707,7 +8723,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>and Electronics Engineering Bachelor of Telecommunication</t>
+          <t>Bachelor of and Electronics Engineering Telecommunication</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -8950,7 +8966,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Management Bachelor of Community</t>
+          <t>Bachelor of Management Community</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -8977,7 +8993,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Development Bachelor Degree in Human Resource</t>
+          <t>Bachelor Degree in Development Human Resource</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -9004,7 +9020,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree</t>
+          <t>Bachelor Degree Management</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -9031,17 +9047,17 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Mathematics and</t>
+          <t>Bachelor of Science in Mathematics and Bachelor of Science with Statistics</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>MAR001</t>
+          <t>MAR001 MAR009</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Two principal passes one of which must be Advanced Mathematics and the other Geography,</t>
+          <t>Two principal passes one of which must be Advanced Mathematics and the other Geography, Economics, Computer Science, Physics, Chemistry. Two principal passes in the following subjects:</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -9058,17 +9074,17 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Education Bachelor of Arts with</t>
+          <t>Bachelor of Arts with Education Bachelor of Arts in Education Economics and Applied Statistics</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>MAR010</t>
+          <t>MAR010 MAR011</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Physics, Advanced Mathematics, Geography, Chemistry or Biology. Two principal passes in the following subjects:</t>
+          <t>Physics, Advanced Mathematics, Geography, Chemistry or Biology. Two principal passes in the following subjects: History, Geography, Kiswahili, Advanced Mathematics, Economics or English. Two principal passes in the following subjects: Advanced Mathematics, Economics, Geography, History, Commerce, Accountancy, Physics, Chemistry or Biology. If one of the principal passes is not in Advanced Mathematics an applicant must have at least a subsidiary pass in Advanced Mathematics or Basic Applied</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -9193,7 +9209,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Engineering Bachelor of Computer</t>
+          <t>Bachelor of Engineering Computer</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -9220,7 +9236,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Engineering and Technology Bachelor of Science with Education</t>
+          <t>Bachelor of Science Engineering and Technology with Education</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -9274,7 +9290,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Technology Bachelor of Science in</t>
+          <t>Bachelor of Science Technology in</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -9301,7 +9317,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Telecommunication Engineering Bachelor of</t>
+          <t>Bachelor of Telecommunication Engineering</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -9382,7 +9398,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Electronics Engineering Bachelor of Technical Education</t>
+          <t>Bachelor of Electronics Engineering Technical Education</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -9409,7 +9425,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>in Mechanical Engineering Bachelor of Technical Education</t>
+          <t>Bachelor of in Mechanical Engineering Technical Education</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -9436,7 +9452,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>in Civil Engineering Bachelor of Technical Education in Architectural</t>
+          <t>Bachelor of in Civil Engineering Technical Education in Architectural</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -9490,7 +9506,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Architecture Bachelor of Engineering in Data Science</t>
+          <t>Bachelor of Architecture Engineering in Data Science</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -9635,7 +9651,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>Chemistry/Biochemistry and Physics Two principal passes of at least ‘ D ’ grade at Advanced Level in Mathematics, Biology and Chemistry or Physics. OR Diploma in Food Sciences and Technology, Laboratory Science and</t>
+          <t>Chemistry/Biochemistry and Physics Two principal passes of at least ‘ D ’ grade at Advanced Level in Mathematics, Biology and Chemistry or Physics. OR Diploma in Food Sciences and Technology, Laboratory Science and applicant must have a minimum of “D” grade in one of the following subjects: Physics, Geography,</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -9814,7 +9830,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Planning Bachelor of Applied Informatics in Industrial Automation</t>
+          <t>Bachelor of Applied Planning Informatics in Industrial Automation</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -9868,7 +9884,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Computer Science Bachelor of Electrical and Electronics</t>
+          <t>Bachelor of Electrical Computer Science and Electronics</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -9895,7 +9911,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Engineering Bachelor of Science in</t>
+          <t>Bachelor of Science in Engineering Engineering</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -9905,7 +9921,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>Chemistry or Geography. Two principalpassesof at least “D”grade at Advanced</t>
+          <t>Chemistry or Geography. Two principalpassesof at least “D”grade at Advanced Geography / Computer Science must have a Credit at</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -9949,7 +9965,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Technology Bachelor of Science in Mechatronics Engineering</t>
+          <t>Bachelor of Science in Technology Mechatronics Engineering</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -10003,7 +10019,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Electrical and Renewable Energy</t>
+          <t>Bachelor of Science in Electrical and Renewable Energy Technology</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -10013,7 +10029,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>“ ” Two pri“nc”ipal passes of at least D grade at Advanced Level in Mathematics and Physics with at least an E grade in Chemistry or Geography.</t>
+          <t>“ ” Two pri“nc”ipal passes of at least D grade at Advanced Level in Mathematics and Physics with at least an E grade in Chemistry or Geography. “ ” “ ”</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -10030,7 +10046,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Control Engineering Bachelor of Science in Information and Computer Networking</t>
+          <t>Bachelor of Science in Control Engineering Information and Computer Networking</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -10300,7 +10316,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Management Bachelor of Accounting and</t>
+          <t>Bachelor of Management Accounting and</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -10327,7 +10343,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Finance Bachelor of Human Resources Management</t>
+          <t>Bachelor of Human Finance Resources Management</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -10435,7 +10451,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Communication Technology Bachelor of Laws</t>
+          <t>Bachelor of Laws Communication Technology</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -10597,7 +10613,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>Pharmacy Bachelor of Science in Environmental Health Sciences</t>
+          <t>Bachelor of Pharmacy Science in Environmental Health Sciences</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -10705,7 +10721,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Surgery Doctor of Medicine</t>
+          <t>Doctor of Medicine Surgery</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -10813,7 +10829,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Laboratory Sciences Bachelor of Science in Audiology and</t>
+          <t>Bachelor of Laboratory Sciences Science in Audiology and</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -10840,7 +10856,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Speech Language Pathology Bachelor of Science in</t>
+          <t>Bachelor of Speech Language Pathology Science in</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -10867,7 +10883,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Occupational Therapy Bachelor of Science in Dental</t>
+          <t>Bachelor of Occupational Therapy Science in Dental</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
@@ -10894,7 +10910,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Laboratory Technology Bachelor of Science in</t>
+          <t>Bachelor of Laboratory Technology Science in</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -10975,7 +10991,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Education Bachelor of Arts in Mass Communication</t>
+          <t>Bachelor of Arts in Education Mass Communication</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -11164,7 +11180,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Bachelor of Arts in Literature and Language Studies</t>
+          <t>Bachelor of Arts in Literature and Language Studies Kiswahili na Lugha za Kigeni</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -11174,7 +11190,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>a minimum of “D” grade in Mathematics at O-Level. Two principal passes in the following subjects: Kiswahili, English Language, French or Arabic. Whereby one of a principal pass must be in English</t>
+          <t>a minimum of “D” grade in Mathematics at O-Level. Two principal passes in the following subjects: Kiswahili, English Language, French or Arabic. Whereby one of a principal pass must be in English Language. ufaulu wenye wastani wa kuanzia alama D mbili, na moja kati ya hizo iwe ya Kiswahili. Pia awe na ufaulu</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">
@@ -11218,7 +11234,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Development Bachelor Degree in Gender and Development</t>
+          <t>Bachelor Degree in Development Gender and Development</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -11326,7 +11342,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Education in Kiswahili and English Languages Bachelor Degree of</t>
+          <t>Bachelor Degree of Education in Kiswahili and English Languages</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -11353,7 +11369,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Education in Geography and History Bachelor Degree of</t>
+          <t>Bachelor Degree of Education in Geography and History</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -11380,7 +11396,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Geography and Kiswahili Bachelor Degree of</t>
+          <t>Bachelor Degree of Geography and Kiswahili</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -11407,7 +11423,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Education in Geography and English Bachelor Degree of</t>
+          <t>Bachelor Degree of Education in Geography and English</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -11434,7 +11450,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Education in History and English Bachelor Degree of</t>
+          <t>Bachelor Degree of Education in History and English</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -11461,7 +11477,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Education in History and Kiswahili Bachelor Degree in Leadership, Ethics and Governance</t>
+          <t>Bachelor Degree in Education in History and Kiswahili Leadership, Ethics and Governance</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -11542,7 +11558,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Development Bachelor Degree in Gender and Development</t>
+          <t>Bachelor Degree Development in Gender and Development</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -11650,7 +11666,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>English Languages Bachelor Degree of Education in Geography and</t>
+          <t>Bachelor Degree English Languages of Education in Geography and</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -11704,7 +11720,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Geography and Kiswahili Bachelor Degree of Education in</t>
+          <t>Bachelor Degree Geography and Kiswahili of Education in</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -11731,7 +11747,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Geography and English Bachelor Degree of Education in</t>
+          <t>Bachelor Degree Geography and English of Education in</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -11758,7 +11774,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>History and English Bachelor Degree of Education in</t>
+          <t>Bachelor Degree History and English of Education in</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -11839,7 +11855,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Development Bachelor Degree in Economics of</t>
+          <t>Bachelor Degree Development in Economics of</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -11920,7 +11936,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Information Technology Bachelor of Science in Fisheries and</t>
+          <t>Bachelor of Science Information Technology in Fisheries and</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -11947,7 +11963,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Aquaculture Bachelor of Science in Crop Science and Production</t>
+          <t>Bachelor of Science Aquaculture in Crop Science and Production</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -12055,7 +12071,7 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>Education Bachelor of Business Administration and Management</t>
+          <t>Bachelor of Education Business Administration and Management</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -12362,7 +12378,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Economics, Commerce, Accountancy, Physics, Chemistry, Biology or Advanced</t>
+          <t>Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Economics, Commerce, Accountancy, Physics, Chemistry, Biology or Advanced least a subsidiary level pass in Advanced Mathematics or Basic Applied Mathematics at A-level or a minimum of “D” grade in Basic Mathematics and a minimum of ‘D’ grade in English Language at O-Level or a pass in</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
@@ -12439,7 +12455,7 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Human Nutrition, or Geography. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Business Studies, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science</t>
+          <t>Human Nutrition, or Geography. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Business Studies, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science Advanced Mathematics, Economics, Accountancy, Commerce, Business Studies, Physics, Chemistry, Biology, Computer Science, Agriculture, Food and</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
@@ -12493,7 +12509,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>of “C” grade in English and History at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French,</t>
+          <t>of “C” grade in English and History at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Agriculture, Computer Science or Nutrition and one</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
@@ -12547,7 +12563,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>subsidiary. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy,</t>
+          <t>subsidiary. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy, Agriculture, Computer Science, Business studies or Nutrition and one subsidiary. If one of the principals do not include Advanced Mathematics or Economics or “ ” Commerce or Business studies or Computer Science an applicant must have a minimum of C grade in Basic</t>
         </is>
       </c>
       <c r="E452" t="inlineStr">
@@ -12834,7 +12850,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>Bachelor of Public Administration in</t>
+          <t>Bachelor of Public Administration in Management</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -12844,7 +12860,7 @@
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Mathematics at O-Level. Two principal passes in History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics,</t>
+          <t>Mathematics at O-Level. Two principal passes in History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, subsidiary. Where the principal passes do not include English, an applicant MUST HAVE a minimum of “ C ”</t>
         </is>
       </c>
       <c r="E463" t="inlineStr">
@@ -12888,7 +12904,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>Bachelor of</t>
+          <t>Bachelor of Communication Technology with Business</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
@@ -12898,7 +12914,7 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>Mathematics at O-Level. Two principal passes in History, Geography, Kiswahili,</t>
+          <t>Mathematics at O-Level. Two principal passes in History, Geography, Kiswahili, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition and one subsidiary. If one of the principals do not include Advanced Mathematics, an applicant MUST HAVE a subsidiary pass in Basic Applied Mathematics at A- Level AND a minimum of “ C ” grade in Basic</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
@@ -12969,7 +12985,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>Science Bachelor of Science in Industrial Engineering Management</t>
+          <t>Bachelor of Science Science in Industrial Engineering Management</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
@@ -13023,7 +13039,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>Education Bachelor of Public Administration in Youth Development</t>
+          <t>Bachelor of Public Education Administration in Youth Development</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -13050,7 +13066,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>and Leadership Bachelor of Health Systems in Monitoring</t>
+          <t>Bachelor of and Leadership Health Systems in Monitoring and Evaluation Environmental</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -13060,7 +13076,7 @@
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>Two principal passes and one subsidiary at the A ‘level. Where the principal passes do not include English and Mathematics an applicant MUST HAVE obtained at least a credit in English Language and Mathematics at</t>
+          <t>Two principal passes and one subsidiary at the A ‘level. Where the principal passes do not include English and Mathematics an applicant MUST HAVE obtained at least a credit in English Language and Mathematics at ‘O’ level. Geography, Biology, Physics; Agriculture, History E‘conomics, Chemistry, Mathematics. The applicant must have obtained at least a credit in Geography at</t>
         </is>
       </c>
       <c r="E471" t="inlineStr">
@@ -13077,7 +13093,7 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>Bachelor of Transport and Logistics Management</t>
+          <t>Bachelor of Transport and Logistics Management Administration in Customer Service Management and Public Relations</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
@@ -13087,7 +13103,7 @@
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>O' level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science, Business studies or Nutrition and one subsidiary. If one of the principal passes do not include Advanced Mathematics or Economics or Commerce or Business studies or Computer Science, an applicant must have a minimum</t>
+          <t>O' level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science, Business studies or Nutrition and one subsidiary. If one of the principal passes do not include Advanced Mathematics or Economics or Commerce or Business studies or Computer Science, an applicant must have a minimum of “C” grade in Basic Mathematics at O-Level. Language or Literature in English, French, Arabic, Chinese, Fine Arts, Economics, Commerce, Accountancy, Business Studies, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science, Food and Human nutrition, Sport, Music</t>
         </is>
       </c>
       <c r="E472" t="inlineStr">
@@ -13222,7 +13238,7 @@
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>Two principal passes in History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition and one subsidiary. If one of the principals do</t>
+          <t>Two principal passes in History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition and one subsidiary. If one of the principals do grade in Basic Mathematics or Commerce or Book-</t>
         </is>
       </c>
       <c r="E477" t="inlineStr">
@@ -13303,7 +13319,7 @@
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>or Nutrition and one subsidiary A-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science, Business studies or</t>
+          <t>or Nutrition and one subsidiary A-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science, Business studies or Commerce or Business studies or Computer Science an applicant must have a minimum of “C” grade in Basic</t>
         </is>
       </c>
       <c r="E480" t="inlineStr">
@@ -13401,7 +13417,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>in Automobile Engineering Bachelor Degree in Procurement and Logistics Management</t>
+          <t>Bachelor Degree in Automobile Engineering in Procurement and Logistics Management</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
@@ -13509,7 +13525,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>Engineering Bachelor Degree in Business Administration</t>
+          <t>Bachelor Degree Engineering in Business Administration</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -13644,7 +13660,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>in Computer Science Bachelor Degree in Aircraft</t>
+          <t>Bachelor Degree in Computer Science in Aircraft</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
@@ -13671,7 +13687,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>Maintenance Engineering. Bachelor Degree in Road and Railway Transport</t>
+          <t>Bachelor Degree Maintenance Engineering. in Road and Railway Transport Logistics Management Port Logistics Management</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
@@ -13681,7 +13697,7 @@
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>subsidiary pass in Chemistry at A-Level or a minimum of “D” grade in Chemistry at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology,</t>
+          <t>subsidiary pass in Chemistry at A-Level or a minimum of “D” grade in Chemistry at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology,</t>
         </is>
       </c>
       <c r="E494" t="inlineStr">
@@ -13725,7 +13741,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>and Marine Engineering Bachelor Degree in Civil and</t>
+          <t>Bachelor Degree and Marine Engineering in Civil and</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
@@ -13752,7 +13768,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>Railway Engineering Bachelor’s</t>
+          <t>Bachelor’s Railway Engineering Railway</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
@@ -13762,7 +13778,7 @@
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>Two principal passes in Advanced Mathematics,</t>
+          <t>Two principal passes in Advanced Mathematics, Mathematics/ Physics/Engineering Science and</t>
         </is>
       </c>
       <c r="E497" t="inlineStr">
@@ -13779,7 +13795,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>Electrification Engineering Bachelor’s degree in education with</t>
+          <t>Bachelor’s Electrification Engineering degree in education with</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
@@ -13806,7 +13822,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>Economics and Mathematics Bachelor’s degree in Telecommunicat ion and Railway</t>
+          <t>Bachelor’s Economics and Mathematics degree in Telecommunicat ion and Railway</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
@@ -13860,7 +13876,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>Education Bachelor of Arts in Journalism</t>
+          <t>Bachelor of Education Arts in Journalism</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -14130,7 +14146,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>Education Bachelor of Science in ICT</t>
+          <t>Bachelor of Education Science in ICT</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
@@ -14265,7 +14281,7 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>Resource Management) Bachelor of Business Administration (International Business)</t>
+          <t>Bachelor of Resource Management) Business Administration (International Business)</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
@@ -14292,7 +14308,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>Bachelor of Human Resource Management</t>
+          <t>Bachelor of Human Resource Management Management</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -14302,7 +14318,7 @@
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced</t>
+          <t>Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Advanced Mathematics, Agriculture, Computer</t>
         </is>
       </c>
       <c r="E517" t="inlineStr">
@@ -14373,7 +14389,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>Linguistics Bachelor of Arts</t>
+          <t>Bachelor of Arts Linguistics</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -14400,7 +14416,7 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>Studies Bachelor of Arts in Natural Resources Management</t>
+          <t>Bachelor of Studies Arts in Natural Resources Management</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
@@ -14427,7 +14443,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>Bachelor of Arts in Population and Development</t>
+          <t>Bachelor of Arts in Population and Development Administration</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
@@ -14437,7 +14453,7 @@
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>Biology, Advanced Mathematics, Agriculture, Computer Science. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry,</t>
+          <t>Biology, Advanced Mathematics, Agriculture, Computer Science. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science. French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry,</t>
         </is>
       </c>
       <c r="E522" t="inlineStr">
@@ -14670,7 +14686,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>with Education Bachelor of Laws</t>
+          <t>Bachelor of with Education Laws</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
@@ -14724,7 +14740,7 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>Computer Science Bachelor of Business Administration</t>
+          <t>Bachelor of Computer Science Business Administration</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
@@ -14832,7 +14848,7 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>Education (IT and Mathematics) Bachelor of Business</t>
+          <t>Bachelor of Education (IT and Mathematics) Business</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
@@ -14859,7 +14875,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>Administration in accounting Bachelor of Science in Nursing</t>
+          <t>Bachelor of Administration in accounting Science in Nursing</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
@@ -14994,7 +15010,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>in Animal Science and Production Bachelor of Science in Aquaculture</t>
+          <t>Bachelor of Science in Animal Science and Production in Aquaculture</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
@@ -15075,7 +15091,7 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>with Education Bachelor of Science in Environmental Science and Management</t>
+          <t>Bachelor of Science with Education in Environmental Science and Management</t>
         </is>
       </c>
       <c r="C546" t="inlineStr">
@@ -15129,7 +15145,7 @@
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>Science and Technology Bachelor of Science</t>
+          <t>Bachelor of Science Science and Technology</t>
         </is>
       </c>
       <c r="C548" t="inlineStr">
@@ -15156,7 +15172,7 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>in Forestry Bachelor of Science in Horticulture</t>
+          <t>Bachelor of Science in Forestry in Horticulture</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
@@ -15210,7 +15226,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>in Information Technology Bachelor of</t>
+          <t>Bachelor of in Information Technology</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
@@ -15399,7 +15415,7 @@
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>Consumer Studies Bachelor of Information and</t>
+          <t>Bachelor of Consumer Studies Information and</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
@@ -15426,7 +15442,7 @@
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>Records Management Bachelor of Community Development</t>
+          <t>Bachelor of Records Management Community Development</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
@@ -15507,7 +15523,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>Management Bachelor of Development Planning and Management</t>
+          <t>Bachelor of Management Development Planning and Management</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
@@ -15561,7 +15577,7 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>Technologies and Value Addition Bachelor of Science</t>
+          <t>Bachelor of Science Technologies and Value Addition</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
@@ -15588,7 +15604,7 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>in Bee Resources Management Bachelor of Human Resources and Labour Relations Management</t>
+          <t>Bachelor of Human in Bee Resources Management Resources and Labour Relations Management</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
@@ -15669,7 +15685,7 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>Education Bachelor of Horticulture with education</t>
+          <t>Bachelor of Education Horticulture with education</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
@@ -15723,7 +15739,7 @@
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>Catering with Education Bachelor of Aquaculture with</t>
+          <t>Bachelor of Catering with Education Aquaculture with</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
@@ -15750,7 +15766,7 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>Education Bachelor of Livestock</t>
+          <t>Bachelor of Education Livestock</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
@@ -15939,7 +15955,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>Education Bachelor of Arts in Sociology</t>
+          <t>Bachelor of Arts in Education Sociology</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
@@ -15993,7 +16009,7 @@
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>Supply Chain Management Bachelor of Science in Electrical Engineering</t>
+          <t>Bachelor of Science in Supply Chain Management Electrical Engineering</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
@@ -16047,7 +16063,7 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Tourism and</t>
+          <t>Bachelor of Science in Tourism and Hospitality Management</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
@@ -16057,7 +16073,7 @@
       </c>
       <c r="D582" t="inlineStr">
         <is>
-          <t>a subsidiary pass in Chemistry at A-Level or a minimum of “C” grade in Chemistry at O-Level. Two principal passes in the following subjects: Biology, Geography, Chemistry, Physics, History,</t>
+          <t>a subsidiary pass in Chemistry at A-Level or a minimum of “C” grade in Chemistry at O-Level. Two principal passes in the following subjects: Biology, Geography, Chemistry, Physics, History, Agriculture, English, History, Nutrition, Economics or Advanced Mathematics.</t>
         </is>
       </c>
       <c r="E582" t="inlineStr">
@@ -16101,7 +16117,7 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>with Education Bachelor of Science in Tourism</t>
+          <t>Bachelor of with Education Science in Tourism</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
@@ -16236,7 +16252,7 @@
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>Education Bachelor of Science</t>
+          <t>Bachelor of Education Science</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
@@ -16263,7 +16279,7 @@
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>with Education Bachelor of Business Administration</t>
+          <t>Bachelor of with Education Business Administration</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
@@ -16344,7 +16360,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>with Education Bachelor of Accounting</t>
+          <t>Bachelor of with Education Accounting</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -16371,7 +16387,7 @@
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>and Finance Bachelor of Arts in Theology</t>
+          <t>Bachelor of and Finance Arts in Theology</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
@@ -16533,7 +16549,7 @@
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>Technology Bachelor of Science Electrical and</t>
+          <t>Bachelor of Technology Science Electrical and</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -16587,7 +16603,7 @@
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>Telecommunicatio n Engineering Bachelor of Science in Information Systems and</t>
+          <t>Bachelor of Telecommunicatio n Engineering Science in Information Systems and</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -16614,7 +16630,7 @@
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>Network Engineering Bachelor of Science in Mechanical Engineering</t>
+          <t>Bachelor of Network Engineering Science in Mechanical Engineering</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
@@ -16668,7 +16684,7 @@
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>Science with Education Bachelor of</t>
+          <t>Bachelor of Science with Education</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
@@ -16722,7 +16738,7 @@
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>Medicine Bachelor of</t>
+          <t>Bachelor of Medicine</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
@@ -16749,7 +16765,7 @@
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>Science with Education Bachelor of IT Application and Management</t>
+          <t>Bachelor of IT Science with Education Application and Management</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
@@ -16857,7 +16873,7 @@
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>Arts with Education Bachelor Degree in Accounting</t>
+          <t>Bachelor Degree Arts with Education in Accounting</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
@@ -16867,7 +16883,7 @@
       </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>Geography, Kiswahili, English Language or Arabic. Two principal passes in the following subjects: History, Geography, Economics, Commerce,</t>
+          <t>Geography, Kiswahili, English Language or Arabic. Two principal passes in the following subjects: History, Geography, Economics, Commerce, Language, French, Computer Science or Nutrition. If one of the principal passes is not in Advanced Mathematics or Economics, Accountancy or Commerce an applicant MUST HAVE a minimum of</t>
         </is>
       </c>
       <c r="E612" t="inlineStr">
@@ -17100,7 +17116,7 @@
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>Agriculture General Doctor of</t>
+          <t>Doctor of Agriculture General</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
@@ -17127,7 +17143,7 @@
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>Dental Surgery Bachelor of Entrepreneurs hip and Innovation</t>
+          <t>Bachelor of Dental Surgery Entrepreneurs hip and Innovation</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
@@ -17478,7 +17494,7 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Business Administration</t>
+          <t>Bachelor Degree Management in Business Administration</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
@@ -17505,7 +17521,7 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>Bachelor Degree in</t>
+          <t>Bachelor Degree in Finance</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
@@ -17515,7 +17531,7 @@
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Accountancy, Economics, advanced Mathematics,</t>
+          <t>Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Accountancy, Economics, advanced Mathematics, French, Arabic, Nutrition, fine arts, computer science and Kiswahili. If one of the principal passes is not Advanced Mathematics, an applicant MUST HAVE a subsidiary pass in Basic Applied Mathematics at A-Level or a minimum</t>
         </is>
       </c>
       <c r="E636" t="inlineStr">
@@ -17559,7 +17575,7 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>Public Relations Bachelor of Business Development with Entrepreneurs hip</t>
+          <t>Bachelor of Public Relations Business Development with Entrepreneurs hip</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -17694,7 +17710,7 @@
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>Relations Bachelor Degree in Public Sector Accounting and Finance</t>
+          <t>Bachelor Relations Degree in Public Sector Accounting and Finance</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -17825,7 +17841,7 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Marketing and Public relations</t>
+          <t>Bachelor Degree Management in Marketing and Public relations</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
@@ -18068,7 +18084,7 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>Management Bachelor Degree in Human</t>
+          <t>Bachelor Management Degree in Human</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -18095,7 +18111,7 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>Resource Management Bachelor Degree in Marketing and Public Relations</t>
+          <t>Bachelor Resource Management Degree in Marketing and Public Relations</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -18257,7 +18273,7 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>Management Bachelor degree in Human resource Management</t>
+          <t>Bachelor degree in Management Human resource Management</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
@@ -18267,7 +18283,7 @@
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>Computer Science or Food and Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Food and Human Nutrition, Advanced Mathematics, Agriculture, Entrepreneurship, Computer</t>
+          <t>Computer Science or Food and Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Food and Human Nutrition, Advanced Mathematics, Agriculture, Entrepreneurship, Computer Arts, Textile and Garment Construction, Chinees, Education, Business studies, Music, Sports, Fasihi ya Kiswahili, Literature in English, Theatre Arts, Textile and</t>
         </is>
       </c>
       <c r="E664" t="inlineStr">
@@ -18365,17 +18381,17 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>Information Management Bachelor Degree in Secretarial</t>
+          <t>Bachelor Information Management Degree in Secretarial</t>
         </is>
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>TPSD2</t>
+          <t>TPSD2 Code</t>
         </is>
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy,</t>
+          <t>Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Art, Economics, Commerce, Accountancy, Admission Requirements</t>
         </is>
       </c>
       <c r="E668" t="inlineStr">
@@ -18446,7 +18462,7 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>Bachelor Degree in Project</t>
+          <t>Bachelor Degree in Project Development</t>
         </is>
       </c>
       <c r="C671" t="inlineStr">
@@ -18456,7 +18472,7 @@
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili,</t>
+          <t>Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
@@ -18581,17 +18597,17 @@
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>Bachelor of Arts with Education</t>
+          <t>Bachelor of Arts with Education Bachelor of Bachelor of Arts in Social Work Divinity</t>
         </is>
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>TK002</t>
+          <t>TK002 TK007 TK010</t>
         </is>
       </c>
       <c r="D676" t="inlineStr">
         <is>
-          <t>Two principal passes in the following subjects: History, Kiswahili, English or Geography.</t>
+          <t>Two principal passes in the following subjects: History, Kiswahili, English or Geography. Two principal passes in Arts, Science or Business studies. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics,</t>
         </is>
       </c>
       <c r="E676" t="inlineStr">
@@ -18635,7 +18651,7 @@
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>ntal Science. Bachelor of</t>
+          <t>Bachelor of ntal Science.</t>
         </is>
       </c>
       <c r="C678" t="inlineStr">
@@ -18689,7 +18705,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>Science in Computer Science Bachelor of Arts in Economics</t>
+          <t>Bachelor of Arts in Science in Computer Science Economics</t>
         </is>
       </c>
       <c r="C680" t="inlineStr">
@@ -18743,7 +18759,7 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>Human Resource Management Bachelor of Arts in</t>
+          <t>Bachelor of Arts in Human Resource Management</t>
         </is>
       </c>
       <c r="C682" t="inlineStr">
@@ -18770,7 +18786,7 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>Community Development Bachelor of Arts in</t>
+          <t>Bachelor of Arts in Community Development</t>
         </is>
       </c>
       <c r="C683" t="inlineStr">
@@ -18824,7 +18840,7 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>Education Bachelor of Laws</t>
+          <t>Bachelor of Education Laws</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
@@ -18932,7 +18948,7 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>Childhood Education Bachelor of</t>
+          <t>Bachelor of Childhood Education</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
@@ -19067,7 +19083,7 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>and Information Technology Bachelor of Business Administration</t>
+          <t>Bachelor of Business and Information Technology Administration</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
@@ -19094,17 +19110,17 @@
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Business Information Technology</t>
+          <t>Bachelor of Science in Business Information Technology Bachelor of Bachelor of Arts with Education Business Administration in Accounting</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>UN003</t>
+          <t>UN003 UA001 UA002</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>subsidiary pass or a pass in Mathematics at O‟- Level. Two principal passes in the following subjects: Advanced Mathematics, Physics, Chemistry, Biology, and Economics. In addition, for appDlicants without Advanced Mathematics in</t>
+          <t>subsidiary pass or a pass in Mathematics at O‟- Level. Two principal passes in the following subjects: Advanced Mathematics, Physics, Chemistry, Biology, and Economics. In addition, for appDlicants without Advanced Mathematics in Two principal passes in any of the following subjects: Kiswahili, Geography or English. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. If one of the principal passes is not in Advanced Mathematics, an applicant MUST HAVE a subsidiary pass in Basic Applied Mathematics at A- Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. If one of the principals is not in</t>
         </is>
       </c>
       <c r="E695" t="inlineStr">
@@ -19121,17 +19137,17 @@
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>Bachelor of Arts in Religious Studies</t>
+          <t>Bachelor of Arts in Religious Studies Bachelor of Arts Bachelor of Arts in Archaeology in Economics</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>UA008</t>
+          <t>UA008 UD001 UD002</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>History, an applicant MUST HAVE a credit in History or Bible Knowledge at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Divinity, Physics, Chemistry, Biology, Agriculture, Computer Science, Information and Comminication and Technology, Nutrition,</t>
+          <t>History, an applicant MUST HAVE a credit in History or Bible Knowledge at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Divinity, Physics, Chemistry, Biology, Agriculture, Computer Science, Information and Comminication and Technology, Nutrition, Two Principal level passes in Arts and Science subjects. Two principal passes one of which must be in Economics or Advanced Mathematics. Candidates</t>
         </is>
       </c>
       <c r="E696" t="inlineStr">
@@ -19175,7 +19191,7 @@
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>in Archaeology and History Bachelor of Arts in Geography and Environmental Studies</t>
+          <t>Bachelor of Arts in Archaeology and History in Geography and Environmental Studies</t>
         </is>
       </c>
       <c r="C698" t="inlineStr">
@@ -19229,7 +19245,7 @@
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>in Heritage Management Bachelor of Arts in History</t>
+          <t>Bachelor of Arts in Heritage Management in History</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
@@ -19256,7 +19272,7 @@
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>Bachelor of Arts in Language</t>
+          <t>Bachelor of Arts in Language Studies</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
@@ -19266,7 +19282,7 @@
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>Geography, Fine Arts, French or Arabic. Two Principal Passes, one of which must be a minimum of ‘C’ grade in the following subjects:</t>
+          <t>Geography, Fine Arts, French or Arabic. Two Principal Passes, one of which must be a minimum of ‘C’ grade in the following subjects: English Language, Kiswahili, French, Chinese or Arabic.</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
@@ -19283,7 +19299,7 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>Bachelor of Arts in Literature</t>
+          <t>Bachelor of Arts in Literature Science and</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
@@ -19293,7 +19309,7 @@
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Two principal passes one of which must be at “C” grade or above in Kiswahili, English or French</t>
+          <t>Two principal passes one of which must be at “C” grade or above in Kiswahili, English or French Language, French, Arabic, Fine Arts, Economics,</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
@@ -19310,7 +19326,7 @@
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>Public Administration Bachelor of Arts in Sociology</t>
+          <t>Bachelor of Arts Public Administration in Sociology</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
@@ -19337,7 +19353,7 @@
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>Bachelor of</t>
+          <t>Bachelor of Science in Statistics</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
@@ -19347,7 +19363,7 @@
       </c>
       <c r="D704" t="inlineStr">
         <is>
-          <t>French, Arabic, Fine Art, Economics, Commerce, Accountancy or Advanced Mathematics. Two principal passes one must be in Advanced</t>
+          <t>French, Arabic, Fine Art, Economics, Commerce, Accountancy or Advanced Mathematics. Two principal passes one must be in Advanced Mathematics with a minimum of ‘D’ grade Language, French, Arabic, Chinese, Fine Arts, Literature in English, Theatre Arts, Music, Textile and Garment Construction, Islamic Knowledge and</t>
         </is>
       </c>
       <c r="E704" t="inlineStr">
@@ -19391,7 +19407,7 @@
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>Engineering Bachelor of Science in Computer Engineering and</t>
+          <t>Bachelor of Engineering Science in Computer Engineering and</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
@@ -19445,7 +19461,7 @@
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>Mining Engineering Bachelor of Science in Textile Engineering</t>
+          <t>Bachelor of Science Mining Engineering in Textile Engineering</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
@@ -19499,7 +19515,7 @@
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Telecommunications</t>
+          <t>Bachelor of Science in Telecommunications Engineering</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
@@ -19509,7 +19525,7 @@
       </c>
       <c r="D710" t="inlineStr">
         <is>
-          <t>at A-level must have at least “C” grade at CSEE in Mathematics. Two principal passes in Advanced Mathematics and Physics. An applicant without at least a subsidiary pass in Chemistry must have a minimum of “C” grade at O-</t>
+          <t>at A-level must have at least “C” grade at CSEE in Mathematics. Two principal passes in Advanced Mathematics and Physics. An applicant without at least a subsidiary pass in Chemistry must have a minimum of “C” grade at O- Level.</t>
         </is>
       </c>
       <c r="E710" t="inlineStr">
@@ -19526,7 +19542,7 @@
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>Actuarial Sciences Bachelor of</t>
+          <t>Bachelor of Actuarial Sciences</t>
         </is>
       </c>
       <c r="C711" t="inlineStr">
@@ -19553,7 +19569,7 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>Science in Applied Zoology Bachelor of Science in</t>
+          <t>Bachelor of Science in Applied Zoology Science in</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
@@ -19580,7 +19596,7 @@
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>Botanical Sciences Bachelor of</t>
+          <t>Bachelor of Botanical Sciences</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
@@ -19661,7 +19677,7 @@
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>Science in Geology Bachelor of</t>
+          <t>Bachelor of Science in Geology</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
@@ -19688,7 +19704,7 @@
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>Science in Microbiology Bachelor of Science in Molecular</t>
+          <t>Bachelor of Science in Microbiology Science in Molecular Biology and Biotechnology Wildlife Science</t>
         </is>
       </c>
       <c r="C717" t="inlineStr">
@@ -19698,7 +19714,7 @@
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>following subjects: Physics, Chemistry or Advanced Mathematics. Two principal passes in Biology and in one of the following subjects: Physics, Chemistry or Advanced Mathematics.</t>
+          <t>following subjects: Physics, Chemistry or Advanced Mathematics. Two principal passes in Biology and in one of the following subjects: Physics, Chemistry or Advanced Mathematics. Geography or Advanced Mathematics.</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
@@ -19715,7 +19731,7 @@
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>And Conservation Bachelor of</t>
+          <t>Bachelor of And Conservation</t>
         </is>
       </c>
       <c r="C718" t="inlineStr">
@@ -19742,7 +19758,7 @@
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>Science with Education Bachelor of</t>
+          <t>Bachelor of Science with Education</t>
         </is>
       </c>
       <c r="C719" t="inlineStr">
@@ -19769,7 +19785,7 @@
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>Science with Geology Bachelor of</t>
+          <t>Bachelor of Science with Geology Science in Computer Science Electronic</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
@@ -19779,7 +19795,7 @@
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>subjects: Physics, Chemistry, Biology, Geography, Advanced Mathematics or Computer. Two principal passes in the following subjects:</t>
+          <t>subjects: Physics, Chemistry, Biology, Geography, Advanced Mathematics or Computer. Two principal passes in the following subjects: Advanced Mathematics and Physics or Computer Science.</t>
         </is>
       </c>
       <c r="E720" t="inlineStr">
@@ -19796,7 +19812,7 @@
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>Science and Communication Bachelor of Arts in Journalism</t>
+          <t>Bachelor of Arts Science and Communication in Journalism</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -19941,7 +19957,7 @@
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce,</t>
+          <t>or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Computer Science or Nutrition. If one of the principals is not in Advanced Mathematics an applicant MUST HAVE at least a subsidiary pass in</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
@@ -19995,7 +20011,7 @@
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English</t>
+          <t>Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. If one of the principals is not in Advanced Mathematics an applicant MUST HAVE at least a subsidiary pass</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
@@ -20049,7 +20065,7 @@
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Advanced Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce,</t>
+          <t>Advanced Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Computer Science or Nutrition. If one of the principals is not in Advanced Mathematics an applicant MUST HAVE at least a subsidiary pass</t>
         </is>
       </c>
       <c r="E730" t="inlineStr">
@@ -20066,7 +20082,7 @@
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>Bachelor of</t>
+          <t>Bachelor of Early Childhood</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
@@ -20076,7 +20092,7 @@
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>in Advanced Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects:</t>
+          <t>in Advanced Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: Commerce, Accountancy, Physics, Chemistry, Biology,</t>
         </is>
       </c>
       <c r="E731" t="inlineStr">
@@ -20093,7 +20109,7 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>Education Bachelor of Education in Physical Education and Sports Sciences</t>
+          <t>Bachelor of Education Education in Physical Education and Sports Sciences</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
@@ -20157,7 +20173,7 @@
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>HAVE at least subsidiary passes or a minimum of “C” grade in History and English at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer</t>
+          <t>HAVE at least subsidiary passes or a minimum of “C” grade in History and English at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer MUST HAVE at least subsidiary passes or a</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
@@ -20201,7 +20217,7 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>in Economics and Statistics Bachelor of Science in</t>
+          <t>Bachelor of in Economics and Statistics Science in</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
@@ -20228,7 +20244,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Bachelor of Science in</t>
+          <t>Bachelor of Mechanical Engineering Science in</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
@@ -20255,7 +20271,7 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Industrial Engineering Bachelor of Science in</t>
+          <t>Bachelor of Industrial Engineering Science in</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
@@ -20282,7 +20298,7 @@
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>Processing Engineering Bachelor of Science in Civil</t>
+          <t>Bachelor of Processing Engineering Science in Civil</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
@@ -20309,7 +20325,7 @@
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>Engineering Bachelor of Science in</t>
+          <t>Bachelor of Engineering Science in</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
@@ -20336,7 +20352,7 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>Petroleum Geology Bachelor of Science in</t>
+          <t>Bachelor of Petroleum Geology Science in</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
@@ -20363,7 +20379,7 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>Petroleum Engineering Bachelor of Science in Petroleum</t>
+          <t>Bachelor of Petroleum Engineering Science in Petroleum</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
@@ -20417,7 +20433,7 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>Science in Meteorology Bachelor of</t>
+          <t>Bachelor of Science in Meteorology</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
@@ -20444,7 +20460,7 @@
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>Architecture Bachelor of Library and Information Studies</t>
+          <t>Bachelor of Architecture Library and Information Studies</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
@@ -20498,17 +20514,17 @@
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>Bachelor of</t>
+          <t>Bachelor of Bachelor of Arts Social Work</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>UD066</t>
+          <t>UD066 UD067</t>
         </is>
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>Two Principal passes in Arts subjects plus a credit</t>
+          <t>Two Principal passes in Arts subjects plus a credit pass in General Studies at A-level, and credit passes in Biology and Civics at O-level Two Principal passes in Arts or Science subjects</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
@@ -20525,7 +20541,7 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>in Psychology Bachelor of Arts</t>
+          <t>Bachelor of Arts in Psychology</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
@@ -20589,7 +20605,7 @@
       </c>
       <c r="D750" t="inlineStr">
         <is>
-          <t>Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Tourism , Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture,</t>
+          <t>Science or Nutrition. Two principal passes in the following subjects: History, Geography, Kiswahili, English Language, French, Arabic, Tourism , Fine Arts, Economics, Commerce, Accountancy, Physics, Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition.</t>
         </is>
       </c>
       <c r="E750" t="inlineStr">
@@ -20714,7 +20730,7 @@
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>Keeping Science and Technology Bachelor of Science in Agricultural Engineering and</t>
+          <t>Bachelor of Keeping Science and Technology Science in Agricultural Engineering and</t>
         </is>
       </c>
       <c r="C755" t="inlineStr">
@@ -20741,7 +20757,7 @@
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>Mechanisation Bachelor of Science in</t>
+          <t>Bachelor of Mechanisation Science in</t>
         </is>
       </c>
       <c r="C756" t="inlineStr">
@@ -20768,7 +20784,7 @@
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>Quantity Surveying Bachelor of Science in</t>
+          <t>Bachelor of Quantity Surveying Science in Resources</t>
         </is>
       </c>
       <c r="C757" t="inlineStr">
@@ -20795,7 +20811,7 @@
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>Economics and Business Bachelor of Science in Geomatics</t>
+          <t>Bachelor of Economics and Business Science in Geomatics</t>
         </is>
       </c>
       <c r="C758" t="inlineStr">
@@ -20849,7 +20865,7 @@
       </c>
       <c r="B760" t="inlineStr">
         <is>
-          <t>Medicine Bachelor of Arts in Theatre Arts</t>
+          <t>Bachelor of Arts Medicine in Theatre Arts</t>
         </is>
       </c>
       <c r="C760" t="inlineStr">
@@ -20957,7 +20973,7 @@
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>in Archaeology and Geography Bachelor of Science in</t>
+          <t>Bachelor of in Archaeology and Geography Science in</t>
         </is>
       </c>
       <c r="C764" t="inlineStr">
@@ -20984,7 +21000,7 @@
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>Electronics Engineering Bachelor of</t>
+          <t>Bachelor of Electronics Engineering</t>
         </is>
       </c>
       <c r="C765" t="inlineStr">
@@ -21011,7 +21027,7 @@
       </c>
       <c r="B766" t="inlineStr">
         <is>
-          <t>Science in Marine Sciences Bachelor of Arts in Diplomatic</t>
+          <t>Bachelor of Arts Science in Marine Sciences in Diplomatic</t>
         </is>
       </c>
       <c r="C766" t="inlineStr">
@@ -21065,7 +21081,7 @@
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>Mathematics and Statistics Bachelor of Science in Business</t>
+          <t>Bachelor of Mathematics and Statistics Science in Business</t>
         </is>
       </c>
       <c r="C768" t="inlineStr">
@@ -21092,7 +21108,7 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>Information Technology Bachelor of</t>
+          <t>Bachelor of Information Technology</t>
         </is>
       </c>
       <c r="C769" t="inlineStr">
@@ -21119,7 +21135,7 @@
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>Science in Geophysics Bachelor of Science in Geology and</t>
+          <t>Bachelor of Science in Geophysics Science in Geology and</t>
         </is>
       </c>
       <c r="C770" t="inlineStr">
@@ -21200,7 +21216,7 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>Management and Tourism Bachelor of Science in</t>
+          <t>Bachelor of Management and Tourism Science in</t>
         </is>
       </c>
       <c r="C773" t="inlineStr">
@@ -21227,7 +21243,7 @@
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>Physics and Chemistry Bachelor of Science in Applied</t>
+          <t>Bachelor of Physics and Chemistry Science in Applied</t>
         </is>
       </c>
       <c r="C774" t="inlineStr">
@@ -21254,7 +21270,7 @@
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>Microbiology and Chemistry Bachelor of Commerce in Procurement and Supply Chain Management</t>
+          <t>Bachelor of Microbiology and Chemistry Commerce in Procurement and Supply Chain Management</t>
         </is>
       </c>
       <c r="C775" t="inlineStr">
@@ -21335,7 +21351,7 @@
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>Development Bachelor of Science in Physics (Medical</t>
+          <t>Bachelor of Science Development in Physics (Medical</t>
         </is>
       </c>
       <c r="C778" t="inlineStr">
@@ -21416,7 +21432,7 @@
       </c>
       <c r="B781" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Computer Science</t>
+          <t>Bachelor of Science in Computer Science in Information Systems</t>
         </is>
       </c>
       <c r="C781" t="inlineStr">
@@ -21426,7 +21442,7 @@
       </c>
       <c r="D781" t="inlineStr">
         <is>
-          <t>Chemistry and “D” grade in Biology and at least E grade in Physics or Advanced Mathematics. Two principal passes in Advanced Mathematics or Computer Science and one of the following</t>
+          <t>Chemistry and “D” grade in Biology and at least E grade in Physics or Advanced Mathematics. Two principal passes in Advanced Mathematics or Computer Science and one of the following subjects: Physics, Geography, Economics or Chemistry. and one of the following subjects: Physics, Geography, Chemistry, Biology or Computer Science. If one of the principal passes is not in</t>
         </is>
       </c>
       <c r="E781" t="inlineStr">
@@ -21470,7 +21486,7 @@
       </c>
       <c r="B783" t="inlineStr">
         <is>
-          <t>in Software Engineering Bachelor of Information Technology with Business Analytics.</t>
+          <t>Bachelor of in Software Engineering Information Technology with Business Analytics.</t>
         </is>
       </c>
       <c r="C783" t="inlineStr">
@@ -21524,7 +21540,7 @@
       </c>
       <c r="B785" t="inlineStr">
         <is>
-          <t>in Computer Engineering Bachelor of Science in</t>
+          <t>Bachelor of Science in in Computer Engineering</t>
         </is>
       </c>
       <c r="C785" t="inlineStr">
@@ -21551,7 +21567,7 @@
       </c>
       <c r="B786" t="inlineStr">
         <is>
-          <t>Telecommunications Engineering Bachelor of Science</t>
+          <t>Bachelor of Science Telecommunications Engineering</t>
         </is>
       </c>
       <c r="C786" t="inlineStr">
@@ -21578,7 +21594,7 @@
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>in Applied Physics Bachelor of Science</t>
+          <t>Bachelor of Science in Applied Physics</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
@@ -21632,7 +21648,7 @@
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>in Biology Bachelor of Science in Mathematics</t>
+          <t>Bachelor of Science in Biology in Mathematics</t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
@@ -21659,7 +21675,7 @@
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Statistics</t>
+          <t>Bachelor of Science in Statistics in Applied Geology</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
@@ -21669,7 +21685,7 @@
       </c>
       <c r="D790" t="inlineStr">
         <is>
-          <t>Commerce, Accountancy, Physics, Chemistry, or Computer Science. Two principal passes at a minimum of “D” grade in Advanced Mathematics and in one of the following subjects: Geography, Economics,</t>
+          <t>Commerce, Accountancy, Physics, Chemistry, or Computer Science. Two principal passes at a minimum of “D” grade in Advanced Mathematics and in one of the following subjects: Geography, Economics, Commerce, Accountancy, Physics, Chemistry or Advanced Mathematics, Physics, Chemistry, Biology or Geography. In addition, an applicant</t>
         </is>
       </c>
       <c r="E790" t="inlineStr">
@@ -21713,7 +21729,7 @@
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>Engineering Bachelor of Science in Metallurgy and</t>
+          <t>Bachelor of Science Engineering in Metallurgy and</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
@@ -21740,7 +21756,7 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>Mineral Processing Engineering Bachelor of Arts in</t>
+          <t>Bachelor of Arts in Mineral Processing Engineering</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
@@ -21821,7 +21837,7 @@
       </c>
       <c r="B796" t="inlineStr">
         <is>
-          <t>French Bachelor of Arts in</t>
+          <t>Bachelor of Arts in French</t>
         </is>
       </c>
       <c r="C796" t="inlineStr">
@@ -21848,7 +21864,7 @@
       </c>
       <c r="B797" t="inlineStr">
         <is>
-          <t>Tourism and Cultural Heritage Bachelor of Arts in Theatre and Film</t>
+          <t>Bachelor of Arts in Tourism and Cultural Heritage Theatre and Film</t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
@@ -21983,7 +21999,7 @@
       </c>
       <c r="B802" t="inlineStr">
         <is>
-          <t>Political Science and Public Administration Bachelor of Geography and Environmental</t>
+          <t>Bachelor of Political Science and Public Administration Geography and Environmental</t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
@@ -22010,7 +22026,7 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Management Bachelor of Arts in Sociology</t>
+          <t>Bachelor of Arts in Management Sociology</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
@@ -22128,7 +22144,7 @@
       </c>
       <c r="D807" t="inlineStr">
         <is>
-          <t>Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English</t>
+          <t>Mathematics or a minimum of “C” grade in Basic Mathematics at O-Level. Two principal passes in the following subjects: History, Geography, Kiswahili, English Chemistry, Biology, Advanced Mathematics, Agriculture, Computer Science or Nutrition. If one of the principals is not in Advanced Mathematics an applicant MUST HAVE at least a subsidiary</t>
         </is>
       </c>
       <c r="E807" t="inlineStr">
@@ -22253,7 +22269,7 @@
       </c>
       <c r="B812" t="inlineStr">
         <is>
-          <t>Bachelor of Arts in Environmental Economics and Policy</t>
+          <t>Bachelor of Arts in Environmental Economics and Policy Disaster Risk</t>
         </is>
       </c>
       <c r="C812" t="inlineStr">
@@ -22263,7 +22279,7 @@
       </c>
       <c r="D812" t="inlineStr">
         <is>
-          <t>Two principal passes in the following subjects: Physics, Chemistry, Advanced Mathematics, Biology, Geography, Economics, Commerce or Accountancy. If one of the principal passes is not in Advanced Mathematics an applicant MUST HAVE at least a subsidiary pass in Advanced Mathematics or Basic</t>
+          <t>Two principal passes in the following subjects: Physics, Chemistry, Advanced Mathematics, Biology, Geography, Economics, Commerce or Accountancy. If one of the principal passes is not in Advanced Mathematics an applicant MUST HAVE at least a subsidiary pass in Advanced Mathematics or Basic Applied Mathematics or a minimum of “C” grade in of the following subjects: Economics, Agriculture,</t>
         </is>
       </c>
       <c r="E812" t="inlineStr">
@@ -22280,7 +22296,7 @@
       </c>
       <c r="B813" t="inlineStr">
         <is>
-          <t>Management Bachelor of Arts in Development Studies</t>
+          <t>Bachelor of Arts in Management Development Studies</t>
         </is>
       </c>
       <c r="C813" t="inlineStr">
@@ -22317,7 +22333,7 @@
       </c>
       <c r="D814" t="inlineStr">
         <is>
-          <t>Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Physics, Chemistry, Advanced Mathematics, Biology, Geography, Economics, Commerce or Accountancy. If one of the principal passes is not</t>
+          <t>Advanced Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Physics, Chemistry, Advanced Mathematics, Biology, Geography, Economics, Commerce or Accountancy. If one of the principal passes is not Advanced Mathematics or Basic Applied</t>
         </is>
       </c>
       <c r="E814" t="inlineStr">
@@ -22361,7 +22377,7 @@
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>International Relations Bachelor of Laws</t>
+          <t>Bachelor of Laws International Relations</t>
         </is>
       </c>
       <c r="C816" t="inlineStr">
@@ -22550,7 +22566,7 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>Security Engineering Bachelor of Science in Petroleum Engineering</t>
+          <t>Bachelor of Science Security Engineering in Petroleum Engineering</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
@@ -22604,7 +22620,7 @@
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>Political Science Bachelor of Commerce in Procurement and Logistics Management</t>
+          <t>Bachelor of Political Science Commerce in Procurement and Logistics Management</t>
         </is>
       </c>
       <c r="C825" t="inlineStr">
@@ -22685,7 +22701,7 @@
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Language and Culture Bachelor of Science in Instructional Design and</t>
+          <t>Bachelor of Science in Language and Culture Instructional Design and</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
@@ -22712,7 +22728,7 @@
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>Information Technology Bachelor of Science in Multimedia</t>
+          <t>Bachelor of Science in Information Technology Multimedia</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
@@ -22766,7 +22782,7 @@
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>Translation and Interpretation Bachelor of Science</t>
+          <t>Bachelor of Science Translation and Interpretation</t>
         </is>
       </c>
       <c r="C831" t="inlineStr">
@@ -22793,7 +22809,7 @@
       </c>
       <c r="B832" t="inlineStr">
         <is>
-          <t>in Geo-informatics Bachelor of Science in Environmental Engineering</t>
+          <t>Bachelor of Science in Geo-informatics in Environmental Engineering</t>
         </is>
       </c>
       <c r="C832" t="inlineStr">
@@ -22901,7 +22917,7 @@
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>in Aquaculture and Aquatic Sciences Bachelor of Science in Clinical Nutrition and Dietetics</t>
+          <t>Bachelor of Science in in Aquaculture and Aquatic Sciences Clinical Nutrition and Dietetics</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
@@ -23036,7 +23052,7 @@
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>Digital Forensics Engineering Bachelor of Arts in Archaeology and</t>
+          <t>Bachelor of Arts in Digital Forensics Engineering Archaeology and</t>
         </is>
       </c>
       <c r="C841" t="inlineStr">
@@ -23063,7 +23079,7 @@
       </c>
       <c r="B842" t="inlineStr">
         <is>
-          <t>Cultural Anthropology Bachelor of Arts in Journalism and Public Relations</t>
+          <t>Bachelor of Arts Cultural Anthropology in Journalism and Public Relations</t>
         </is>
       </c>
       <c r="C842" t="inlineStr">
@@ -23171,7 +23187,7 @@
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>Kiswahili Bachelor of Pharmacy</t>
+          <t>Bachelor of Kiswahili Pharmacy</t>
         </is>
       </c>
       <c r="C846" t="inlineStr">
@@ -23279,7 +23295,7 @@
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>Tourism Bachelor of Counselling Psychology</t>
+          <t>Bachelor of Tourism Counselling Psychology</t>
         </is>
       </c>
       <c r="C850" t="inlineStr">
@@ -23846,7 +23862,7 @@
       </c>
       <c r="B871" t="inlineStr">
         <is>
-          <t>Accounting &amp; Finance Bachelor of Procurement and</t>
+          <t>Bachelor of Accounting &amp; Finance Procurement and</t>
         </is>
       </c>
       <c r="C871" t="inlineStr">
@@ -23873,7 +23889,7 @@
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>Logistics Management Bachelor of Business Administration in</t>
+          <t>Bachelor of Logistics Management Business Administration in</t>
         </is>
       </c>
       <c r="C872" t="inlineStr">
@@ -23900,7 +23916,7 @@
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>Marketing Bachelor of Science inBusiness Information</t>
+          <t>Bachelor of Science Marketing inBusiness Information</t>
         </is>
       </c>
       <c r="C873" t="inlineStr">
@@ -24062,7 +24078,7 @@
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>Information Technology Bachelor of Science in Telecommunications</t>
+          <t>Bachelor of Science in Information Technology Telecommunications</t>
         </is>
       </c>
       <c r="C879" t="inlineStr">
@@ -24116,7 +24132,7 @@
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>Bachelor of International Relations and Diplomacy</t>
+          <t>Diplomacy Bachelor of International Relations and</t>
         </is>
       </c>
       <c r="C881" t="inlineStr">
@@ -24234,7 +24250,7 @@
       </c>
       <c r="D885" t="inlineStr">
         <is>
-          <t>Knowledge , Biology, Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects:</t>
+          <t>Knowledge , Biology, Mathematics, Agriculture, Computer Science or Nutrition. Two principal passes in the following subjects: Accountancy, Physics, Chemistry, Biology,</t>
         </is>
       </c>
       <c r="E885" t="inlineStr">
@@ -24315,7 +24331,7 @@
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>Information Technology or Advanced Mathematics. Three principal passes in Chemistry, Biology and either Physics or Mathematics, Nutrition,</t>
+          <t>Information Technology or Advanced Mathematics. Three principal passes in Chemistry, Biology and either Physics or Mathematics, Nutrition, Biology and at least E grade in Physics, Advanced</t>
         </is>
       </c>
       <c r="E888" t="inlineStr">

</xml_diff>